<commit_message>
1st commit of new branch
11/4/2025
</commit_message>
<xml_diff>
--- a/Raw Data/single force (15 trials)(tapered and 2x cylindrical)/Validation(1.5)(3tendon).xlsx
+++ b/Raw Data/single force (15 trials)(tapered and 2x cylindrical)/Validation(1.5)(3tendon).xlsx
@@ -5,12 +5,12 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://djpropertycom-my.sharepoint.com/personal/noah_familiajones_org/Documents/Work and Projects/Github/Whisker_Inspired_Sensing_CR/SoRoSim Robots/my_robot(1.5)(3tendon)/10-09-2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://djpropertycom-my.sharepoint.com/personal/noah_familiajones_org/Documents/Work and Projects/Github/Whisker_Inspired_Sensing_CR/Raw Data/single force (15 trials)(tapered and 2x cylindrical)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2231" documentId="8_{DFFD6B0C-681F-42C8-B2E4-5D4B90AAE966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5CF8404-C50B-4539-92A5-7D57054E371E}"/>
+  <xr:revisionPtr revIDLastSave="2241" documentId="8_{DFFD6B0C-681F-42C8-B2E4-5D4B90AAE966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31010650-0FB4-49EA-BE98-3128C985EAC8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="5" xr2:uid="{3D16C37F-3C74-4527-A308-796C339DFE9F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3D16C37F-3C74-4527-A308-796C339DFE9F}"/>
   </bookViews>
   <sheets>
     <sheet name="Proximal Validation (single)" sheetId="8" r:id="rId1"/>
@@ -418,7 +418,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -490,6 +490,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -511,10 +512,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -834,7 +831,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F22B4A24-01F9-43FA-AE7F-5A1710EEAA53}">
-  <dimension ref="A1:Y18"/>
+  <dimension ref="A1:Y36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -2222,6 +2219,438 @@
         <f t="array" ref="M18">AVERAGE(ABS(M3:M17))</f>
         <v>0.28629773457845042</v>
       </c>
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T19" s="31">
+        <f>H3-N3</f>
+        <v>1.847592519846372E-4</v>
+      </c>
+      <c r="U19" s="31">
+        <f t="shared" ref="U19:Y19" si="1">I3-O3</f>
+        <v>4.2102840154825891E-3</v>
+      </c>
+      <c r="V19" s="31">
+        <f t="shared" si="1"/>
+        <v>-3.5332830537174514E-3</v>
+      </c>
+      <c r="W19" s="31">
+        <f t="shared" si="1"/>
+        <v>-7.452349703906902E-3</v>
+      </c>
+      <c r="X19" s="31">
+        <f t="shared" si="1"/>
+        <v>-2.3155923378939628E-2</v>
+      </c>
+      <c r="Y19" s="31">
+        <f t="shared" si="1"/>
+        <v>-3.0356762917084973E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T20" s="31">
+        <f t="shared" ref="T20:T36" si="2">H4-N4</f>
+        <v>-8.0810196232050701E-4</v>
+      </c>
+      <c r="U20" s="31">
+        <f t="shared" ref="U20:U36" si="3">I4-O4</f>
+        <v>7.7707701963152381E-3</v>
+      </c>
+      <c r="V20" s="31">
+        <f t="shared" ref="V20:V36" si="4">J4-P4</f>
+        <v>4.5860621232501919E-4</v>
+      </c>
+      <c r="W20" s="31">
+        <f t="shared" ref="W20:W36" si="5">K4-Q4</f>
+        <v>1.9074732525887123E-2</v>
+      </c>
+      <c r="X20" s="31">
+        <f t="shared" ref="X20:X36" si="6">L4-R4</f>
+        <v>1.2532535927168194E-3</v>
+      </c>
+      <c r="Y20" s="31">
+        <f t="shared" ref="Y20:Y36" si="7">M4-S4</f>
+        <v>-4.3861778587547806E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T21" s="31">
+        <f t="shared" si="2"/>
+        <v>2.3527816318886039E-3</v>
+      </c>
+      <c r="U21" s="31">
+        <f t="shared" si="3"/>
+        <v>5.4421231823428562E-3</v>
+      </c>
+      <c r="V21" s="31">
+        <f t="shared" si="4"/>
+        <v>-2.2929285054362179E-2</v>
+      </c>
+      <c r="W21" s="31">
+        <f t="shared" si="5"/>
+        <v>-3.4040360368839506E-2</v>
+      </c>
+      <c r="X21" s="31">
+        <f t="shared" si="6"/>
+        <v>-0.10064819745733566</v>
+      </c>
+      <c r="Y21" s="31">
+        <f t="shared" si="7"/>
+        <v>-4.1193938998757673E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T22" s="31">
+        <f t="shared" si="2"/>
+        <v>4.4326256918706146E-4</v>
+      </c>
+      <c r="U22" s="31">
+        <f t="shared" si="3"/>
+        <v>3.7358667806700191E-3</v>
+      </c>
+      <c r="V22" s="31">
+        <f t="shared" si="4"/>
+        <v>-6.7064575228130961E-4</v>
+      </c>
+      <c r="W22" s="31">
+        <f t="shared" si="5"/>
+        <v>5.4523667412911744E-3</v>
+      </c>
+      <c r="X22" s="31">
+        <f t="shared" si="6"/>
+        <v>-9.5033798066236734E-3</v>
+      </c>
+      <c r="Y22" s="31">
+        <f t="shared" si="7"/>
+        <v>-4.4884785550945883E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T23" s="31">
+        <f t="shared" si="2"/>
+        <v>-5.5839424021542105E-4</v>
+      </c>
+      <c r="U23" s="31">
+        <f t="shared" si="3"/>
+        <v>1.3647159970116327E-2</v>
+      </c>
+      <c r="V23" s="31">
+        <f t="shared" si="4"/>
+        <v>-9.6356951723947906E-4</v>
+      </c>
+      <c r="W23" s="31">
+        <f t="shared" si="5"/>
+        <v>5.0590860214492495E-3</v>
+      </c>
+      <c r="X23" s="31">
+        <f t="shared" si="6"/>
+        <v>-2.4432117554092593E-3</v>
+      </c>
+      <c r="Y23" s="31">
+        <f t="shared" si="7"/>
+        <v>-0.10840252226451574</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T24" s="31">
+        <f t="shared" si="2"/>
+        <v>2.2627546639204903E-3</v>
+      </c>
+      <c r="U24" s="31">
+        <f t="shared" si="3"/>
+        <v>9.393346071372155E-3</v>
+      </c>
+      <c r="V24" s="31">
+        <f t="shared" si="4"/>
+        <v>-6.3112483737577871E-3</v>
+      </c>
+      <c r="W24" s="31">
+        <f t="shared" si="5"/>
+        <v>3.7361640346390557E-3</v>
+      </c>
+      <c r="X24" s="31">
+        <f t="shared" si="6"/>
+        <v>-2.4747759349922009E-2</v>
+      </c>
+      <c r="Y24" s="31">
+        <f t="shared" si="7"/>
+        <v>-9.1080466142032246E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T25" s="31">
+        <f t="shared" si="2"/>
+        <v>-5.38935419172049E-4</v>
+      </c>
+      <c r="U25" s="31">
+        <f t="shared" si="3"/>
+        <v>1.730476735149622E-2</v>
+      </c>
+      <c r="V25" s="31">
+        <f t="shared" si="4"/>
+        <v>3.5026456678283512E-3</v>
+      </c>
+      <c r="W25" s="31">
+        <f t="shared" si="5"/>
+        <v>4.5338056478765654E-2</v>
+      </c>
+      <c r="X25" s="31">
+        <f t="shared" si="6"/>
+        <v>1.5648685776274335E-2</v>
+      </c>
+      <c r="Y25" s="31">
+        <f t="shared" si="7"/>
+        <v>-0.10715854673635526</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T26" s="31">
+        <f t="shared" si="2"/>
+        <v>-7.8150304034352292E-4</v>
+      </c>
+      <c r="U26" s="31">
+        <f t="shared" si="3"/>
+        <v>5.543048377637444E-3</v>
+      </c>
+      <c r="V26" s="31">
+        <f t="shared" si="4"/>
+        <v>-1.3857872030263854E-2</v>
+      </c>
+      <c r="W26" s="31">
+        <f t="shared" si="5"/>
+        <v>3.3242495503211344E-2</v>
+      </c>
+      <c r="X26" s="31">
+        <f t="shared" si="6"/>
+        <v>-9.2624964851503067E-2</v>
+      </c>
+      <c r="Y26" s="31">
+        <f t="shared" si="7"/>
+        <v>-3.3466802983233901E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T27" s="31">
+        <f t="shared" si="2"/>
+        <v>-4.8895599320530978E-4</v>
+      </c>
+      <c r="U27" s="31">
+        <f t="shared" si="3"/>
+        <v>9.3275129724849221E-4</v>
+      </c>
+      <c r="V27" s="31">
+        <f t="shared" si="4"/>
+        <v>-4.708825375822151E-3</v>
+      </c>
+      <c r="W27" s="31">
+        <f t="shared" si="5"/>
+        <v>1.4616601539097773E-2</v>
+      </c>
+      <c r="X27" s="31">
+        <f t="shared" si="6"/>
+        <v>-1.9879507525760454E-2</v>
+      </c>
+      <c r="Y27" s="31">
+        <f t="shared" si="7"/>
+        <v>1.5558310962285327E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T28" s="31">
+        <f t="shared" si="2"/>
+        <v>1.6981890338156414E-3</v>
+      </c>
+      <c r="U28" s="31">
+        <f t="shared" si="3"/>
+        <v>-1.0251584254363608E-2</v>
+      </c>
+      <c r="V28" s="31">
+        <f t="shared" si="4"/>
+        <v>2.1096944113437238E-2</v>
+      </c>
+      <c r="W28" s="31">
+        <f t="shared" si="5"/>
+        <v>0.27340172303897181</v>
+      </c>
+      <c r="X28" s="31">
+        <f t="shared" si="6"/>
+        <v>4.8363402659864385E-2</v>
+      </c>
+      <c r="Y28" s="31">
+        <f t="shared" si="7"/>
+        <v>2.9085556228708065E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T29" s="31">
+        <f t="shared" si="2"/>
+        <v>1.0726011326152585E-3</v>
+      </c>
+      <c r="U29" s="31">
+        <f t="shared" si="3"/>
+        <v>-4.7009595893940312E-3</v>
+      </c>
+      <c r="V29" s="31">
+        <f t="shared" si="4"/>
+        <v>1.178789845857954E-2</v>
+      </c>
+      <c r="W29" s="31">
+        <f t="shared" si="5"/>
+        <v>1.2331545464643906E-2</v>
+      </c>
+      <c r="X29" s="31">
+        <f t="shared" si="6"/>
+        <v>6.7203509450865118E-2</v>
+      </c>
+      <c r="Y29" s="31">
+        <f t="shared" si="7"/>
+        <v>3.7628630027377041E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T30" s="31">
+        <f t="shared" si="2"/>
+        <v>-4.8972228571948458E-4</v>
+      </c>
+      <c r="U30" s="31">
+        <f t="shared" si="3"/>
+        <v>-5.2178100793420987E-3</v>
+      </c>
+      <c r="V30" s="31">
+        <f t="shared" si="4"/>
+        <v>7.1161220757140556E-3</v>
+      </c>
+      <c r="W30" s="31">
+        <f t="shared" si="5"/>
+        <v>2.145602025424935E-2</v>
+      </c>
+      <c r="X30" s="31">
+        <f t="shared" si="6"/>
+        <v>5.3121850748457711E-2</v>
+      </c>
+      <c r="Y30" s="31">
+        <f t="shared" si="7"/>
+        <v>3.8358183479932639E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T31" s="31">
+        <f t="shared" si="2"/>
+        <v>-1.6191133978591887E-4</v>
+      </c>
+      <c r="U31" s="31">
+        <f t="shared" si="3"/>
+        <v>7.3863404524286691E-4</v>
+      </c>
+      <c r="V31" s="31">
+        <f t="shared" si="4"/>
+        <v>-4.576913807206151E-3</v>
+      </c>
+      <c r="W31" s="31">
+        <f t="shared" si="5"/>
+        <v>-2.7453060663472056E-2</v>
+      </c>
+      <c r="X31" s="31">
+        <f t="shared" si="6"/>
+        <v>1.2478955333677488E-2</v>
+      </c>
+      <c r="Y31" s="31">
+        <f t="shared" si="7"/>
+        <v>2.2424507352374223E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="T32" s="31">
+        <f t="shared" si="2"/>
+        <v>3.2763835042714964E-4</v>
+      </c>
+      <c r="U32" s="31">
+        <f t="shared" si="3"/>
+        <v>-5.7683251419953993E-3</v>
+      </c>
+      <c r="V32" s="31">
+        <f t="shared" si="4"/>
+        <v>9.8612683599342277E-3</v>
+      </c>
+      <c r="W32" s="31">
+        <f t="shared" si="5"/>
+        <v>2.2872080768403247E-2</v>
+      </c>
+      <c r="X32" s="31">
+        <f t="shared" si="6"/>
+        <v>6.3356841061008973E-2</v>
+      </c>
+      <c r="Y32" s="31">
+        <f t="shared" si="7"/>
+        <v>3.7839914167488053E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="20:25" x14ac:dyDescent="0.25">
+      <c r="T33" s="31">
+        <f t="shared" si="2"/>
+        <v>3.5051628947257974E-4</v>
+      </c>
+      <c r="U33" s="31">
+        <f t="shared" si="3"/>
+        <v>-6.3251123980629306E-3</v>
+      </c>
+      <c r="V33" s="31">
+        <f t="shared" si="4"/>
+        <v>1.2023195374459394E-2</v>
+      </c>
+      <c r="W33" s="31">
+        <f t="shared" si="5"/>
+        <v>3.0015087212819286E-2</v>
+      </c>
+      <c r="X33" s="31">
+        <f t="shared" si="6"/>
+        <v>6.6442767616919279E-2</v>
+      </c>
+      <c r="Y33" s="31">
+        <f t="shared" si="7"/>
+        <v>3.6352825687667525E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="20:25" x14ac:dyDescent="0.25">
+      <c r="T34" s="31"/>
+      <c r="U34" s="31"/>
+      <c r="V34" s="31"/>
+      <c r="W34" s="31"/>
+      <c r="X34" s="31"/>
+      <c r="Y34" s="31"/>
+    </row>
+    <row r="35" spans="20:25" x14ac:dyDescent="0.25">
+      <c r="T35" s="31">
+        <f>_xlfn.STDEV.S(T19:T33)</f>
+        <v>1.0671748468220961E-3</v>
+      </c>
+      <c r="U35" s="31">
+        <f t="shared" ref="U35:Y35" si="8">_xlfn.STDEV.S(U19:U33)</f>
+        <v>7.8688500421000025E-3</v>
+      </c>
+      <c r="V35" s="31">
+        <f t="shared" si="8"/>
+        <v>1.1016145258516748E-2</v>
+      </c>
+      <c r="W35" s="31">
+        <f t="shared" si="8"/>
+        <v>7.1179610812383928E-2</v>
+      </c>
+      <c r="X35" s="31">
+        <f t="shared" si="8"/>
+        <v>5.2547292552495489E-2</v>
+      </c>
+      <c r="Y35" s="31">
+        <f t="shared" si="8"/>
+        <v>5.3660086491622155E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="20:25" x14ac:dyDescent="0.25">
+      <c r="T36" s="31"/>
+      <c r="U36" s="31"/>
+      <c r="V36" s="31"/>
+      <c r="W36" s="31"/>
+      <c r="X36" s="31"/>
+      <c r="Y36" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -26962,12 +27391,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="W2:Y2"/>
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="H2:M2"/>
     <mergeCell ref="N2:R2"/>
     <mergeCell ref="S2:U2"/>
-    <mergeCell ref="W2:Y2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -40426,12 +40855,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -40688,17 +41116,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D595912-0053-4104-933F-CDA3B3DBC546}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE208467-E14A-4CB9-9FC8-72DFB8E94FF2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -40723,18 +41161,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE208467-E14A-4CB9-9FC8-72DFB8E94FF2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D595912-0053-4104-933F-CDA3B3DBC546}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Pre topology opt + purterbations
11/5/2025
</commit_message>
<xml_diff>
--- a/Raw Data/single force (15 trials)(tapered and 2x cylindrical)/Validation(1.5)(3tendon).xlsx
+++ b/Raw Data/single force (15 trials)(tapered and 2x cylindrical)/Validation(1.5)(3tendon).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://djpropertycom-my.sharepoint.com/personal/noah_familiajones_org/Documents/Work and Projects/Github/Whisker_Inspired_Sensing_CR/Raw Data/single force (15 trials)(tapered and 2x cylindrical)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2241" documentId="8_{DFFD6B0C-681F-42C8-B2E4-5D4B90AAE966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31010650-0FB4-49EA-BE98-3128C985EAC8}"/>
+  <xr:revisionPtr revIDLastSave="2246" documentId="8_{DFFD6B0C-681F-42C8-B2E4-5D4B90AAE966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8A8B0D0-E12A-4407-83D4-863216286743}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3D16C37F-3C74-4527-A308-796C339DFE9F}"/>
   </bookViews>
@@ -436,6 +436,7 @@
     <xf numFmtId="11" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="9" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -490,7 +491,6 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -512,6 +512,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -838,39 +842,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="15" t="s">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="17" t="s">
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
-      <c r="S1" s="18"/>
-      <c r="T1" s="19" t="s">
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
+      <c r="S1" s="19"/>
+      <c r="T1" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="20"/>
-      <c r="V1" s="20"/>
-      <c r="W1" s="20"/>
-      <c r="X1" s="20"/>
-      <c r="Y1" s="21"/>
+      <c r="U1" s="21"/>
+      <c r="V1" s="21"/>
+      <c r="W1" s="21"/>
+      <c r="X1" s="21"/>
+      <c r="Y1" s="22"/>
     </row>
     <row r="2" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2221,436 +2225,440 @@
       </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T19" s="31">
+      <c r="T19" s="13">
         <f>H3-N3</f>
         <v>1.847592519846372E-4</v>
       </c>
-      <c r="U19" s="31">
+      <c r="U19" s="13">
         <f t="shared" ref="U19:Y19" si="1">I3-O3</f>
         <v>4.2102840154825891E-3</v>
       </c>
-      <c r="V19" s="31">
+      <c r="V19" s="13">
         <f t="shared" si="1"/>
         <v>-3.5332830537174514E-3</v>
       </c>
-      <c r="W19" s="31">
+      <c r="W19" s="13">
         <f t="shared" si="1"/>
         <v>-7.452349703906902E-3</v>
       </c>
-      <c r="X19" s="31">
+      <c r="X19" s="13">
         <f t="shared" si="1"/>
         <v>-2.3155923378939628E-2</v>
       </c>
-      <c r="Y19" s="31">
+      <c r="Y19" s="13">
         <f t="shared" si="1"/>
         <v>-3.0356762917084973E-2</v>
       </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T20" s="31">
-        <f t="shared" ref="T20:T36" si="2">H4-N4</f>
+      <c r="T20" s="13">
+        <f t="shared" ref="T20:T33" si="2">H4-N4</f>
         <v>-8.0810196232050701E-4</v>
       </c>
-      <c r="U20" s="31">
-        <f t="shared" ref="U20:U36" si="3">I4-O4</f>
+      <c r="U20" s="13">
+        <f t="shared" ref="U20:U33" si="3">I4-O4</f>
         <v>7.7707701963152381E-3</v>
       </c>
-      <c r="V20" s="31">
-        <f t="shared" ref="V20:V36" si="4">J4-P4</f>
+      <c r="V20" s="13">
+        <f t="shared" ref="V20:V33" si="4">J4-P4</f>
         <v>4.5860621232501919E-4</v>
       </c>
-      <c r="W20" s="31">
-        <f t="shared" ref="W20:W36" si="5">K4-Q4</f>
+      <c r="W20" s="13">
+        <f t="shared" ref="W20:W33" si="5">K4-Q4</f>
         <v>1.9074732525887123E-2</v>
       </c>
-      <c r="X20" s="31">
-        <f t="shared" ref="X20:X36" si="6">L4-R4</f>
+      <c r="X20" s="13">
+        <f t="shared" ref="X20:X33" si="6">L4-R4</f>
         <v>1.2532535927168194E-3</v>
       </c>
-      <c r="Y20" s="31">
-        <f t="shared" ref="Y20:Y36" si="7">M4-S4</f>
+      <c r="Y20" s="13">
+        <f t="shared" ref="Y20:Y33" si="7">M4-S4</f>
         <v>-4.3861778587547806E-2</v>
       </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T21" s="31">
+      <c r="T21" s="13">
         <f t="shared" si="2"/>
         <v>2.3527816318886039E-3</v>
       </c>
-      <c r="U21" s="31">
+      <c r="U21" s="13">
         <f t="shared" si="3"/>
         <v>5.4421231823428562E-3</v>
       </c>
-      <c r="V21" s="31">
+      <c r="V21" s="13">
         <f t="shared" si="4"/>
         <v>-2.2929285054362179E-2</v>
       </c>
-      <c r="W21" s="31">
+      <c r="W21" s="13">
         <f t="shared" si="5"/>
         <v>-3.4040360368839506E-2</v>
       </c>
-      <c r="X21" s="31">
+      <c r="X21" s="13">
         <f t="shared" si="6"/>
         <v>-0.10064819745733566</v>
       </c>
-      <c r="Y21" s="31">
+      <c r="Y21" s="13">
         <f t="shared" si="7"/>
         <v>-4.1193938998757673E-2</v>
       </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T22" s="31">
+      <c r="T22" s="13">
         <f t="shared" si="2"/>
         <v>4.4326256918706146E-4</v>
       </c>
-      <c r="U22" s="31">
+      <c r="U22" s="13">
         <f t="shared" si="3"/>
         <v>3.7358667806700191E-3</v>
       </c>
-      <c r="V22" s="31">
+      <c r="V22" s="13">
         <f t="shared" si="4"/>
         <v>-6.7064575228130961E-4</v>
       </c>
-      <c r="W22" s="31">
+      <c r="W22" s="13">
         <f t="shared" si="5"/>
         <v>5.4523667412911744E-3</v>
       </c>
-      <c r="X22" s="31">
+      <c r="X22" s="13">
         <f t="shared" si="6"/>
         <v>-9.5033798066236734E-3</v>
       </c>
-      <c r="Y22" s="31">
+      <c r="Y22" s="13">
         <f t="shared" si="7"/>
         <v>-4.4884785550945883E-2</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T23" s="31">
+      <c r="T23" s="13">
         <f t="shared" si="2"/>
         <v>-5.5839424021542105E-4</v>
       </c>
-      <c r="U23" s="31">
+      <c r="U23" s="13">
         <f t="shared" si="3"/>
         <v>1.3647159970116327E-2</v>
       </c>
-      <c r="V23" s="31">
+      <c r="V23" s="13">
         <f t="shared" si="4"/>
         <v>-9.6356951723947906E-4</v>
       </c>
-      <c r="W23" s="31">
+      <c r="W23" s="13">
         <f t="shared" si="5"/>
         <v>5.0590860214492495E-3</v>
       </c>
-      <c r="X23" s="31">
+      <c r="X23" s="13">
         <f t="shared" si="6"/>
         <v>-2.4432117554092593E-3</v>
       </c>
-      <c r="Y23" s="31">
+      <c r="Y23" s="13">
         <f t="shared" si="7"/>
         <v>-0.10840252226451574</v>
       </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T24" s="31">
+      <c r="T24" s="13">
         <f t="shared" si="2"/>
         <v>2.2627546639204903E-3</v>
       </c>
-      <c r="U24" s="31">
+      <c r="U24" s="13">
         <f t="shared" si="3"/>
         <v>9.393346071372155E-3</v>
       </c>
-      <c r="V24" s="31">
+      <c r="V24" s="13">
         <f t="shared" si="4"/>
         <v>-6.3112483737577871E-3</v>
       </c>
-      <c r="W24" s="31">
+      <c r="W24" s="13">
         <f t="shared" si="5"/>
         <v>3.7361640346390557E-3</v>
       </c>
-      <c r="X24" s="31">
+      <c r="X24" s="13">
         <f t="shared" si="6"/>
         <v>-2.4747759349922009E-2</v>
       </c>
-      <c r="Y24" s="31">
+      <c r="Y24" s="13">
         <f t="shared" si="7"/>
         <v>-9.1080466142032246E-2</v>
       </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T25" s="31">
+      <c r="T25" s="13">
         <f t="shared" si="2"/>
         <v>-5.38935419172049E-4</v>
       </c>
-      <c r="U25" s="31">
+      <c r="U25" s="13">
         <f t="shared" si="3"/>
         <v>1.730476735149622E-2</v>
       </c>
-      <c r="V25" s="31">
+      <c r="V25" s="13">
         <f t="shared" si="4"/>
         <v>3.5026456678283512E-3</v>
       </c>
-      <c r="W25" s="31">
+      <c r="W25" s="13">
         <f t="shared" si="5"/>
         <v>4.5338056478765654E-2</v>
       </c>
-      <c r="X25" s="31">
+      <c r="X25" s="13">
         <f t="shared" si="6"/>
         <v>1.5648685776274335E-2</v>
       </c>
-      <c r="Y25" s="31">
+      <c r="Y25" s="13">
         <f t="shared" si="7"/>
         <v>-0.10715854673635526</v>
       </c>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T26" s="31">
+      <c r="G26">
+        <f>N23</f>
+        <v>0</v>
+      </c>
+      <c r="T26" s="13">
         <f t="shared" si="2"/>
         <v>-7.8150304034352292E-4</v>
       </c>
-      <c r="U26" s="31">
+      <c r="U26" s="13">
         <f t="shared" si="3"/>
         <v>5.543048377637444E-3</v>
       </c>
-      <c r="V26" s="31">
+      <c r="V26" s="13">
         <f t="shared" si="4"/>
         <v>-1.3857872030263854E-2</v>
       </c>
-      <c r="W26" s="31">
+      <c r="W26" s="13">
         <f t="shared" si="5"/>
         <v>3.3242495503211344E-2</v>
       </c>
-      <c r="X26" s="31">
+      <c r="X26" s="13">
         <f t="shared" si="6"/>
         <v>-9.2624964851503067E-2</v>
       </c>
-      <c r="Y26" s="31">
+      <c r="Y26" s="13">
         <f t="shared" si="7"/>
         <v>-3.3466802983233901E-2</v>
       </c>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T27" s="31">
+      <c r="T27" s="13">
         <f t="shared" si="2"/>
         <v>-4.8895599320530978E-4</v>
       </c>
-      <c r="U27" s="31">
+      <c r="U27" s="13">
         <f t="shared" si="3"/>
         <v>9.3275129724849221E-4</v>
       </c>
-      <c r="V27" s="31">
+      <c r="V27" s="13">
         <f t="shared" si="4"/>
         <v>-4.708825375822151E-3</v>
       </c>
-      <c r="W27" s="31">
+      <c r="W27" s="13">
         <f t="shared" si="5"/>
         <v>1.4616601539097773E-2</v>
       </c>
-      <c r="X27" s="31">
+      <c r="X27" s="13">
         <f t="shared" si="6"/>
         <v>-1.9879507525760454E-2</v>
       </c>
-      <c r="Y27" s="31">
+      <c r="Y27" s="13">
         <f t="shared" si="7"/>
         <v>1.5558310962285327E-3</v>
       </c>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T28" s="31">
+      <c r="T28" s="13">
         <f t="shared" si="2"/>
         <v>1.6981890338156414E-3</v>
       </c>
-      <c r="U28" s="31">
+      <c r="U28" s="13">
         <f t="shared" si="3"/>
         <v>-1.0251584254363608E-2</v>
       </c>
-      <c r="V28" s="31">
+      <c r="V28" s="13">
         <f t="shared" si="4"/>
         <v>2.1096944113437238E-2</v>
       </c>
-      <c r="W28" s="31">
+      <c r="W28" s="13">
         <f t="shared" si="5"/>
         <v>0.27340172303897181</v>
       </c>
-      <c r="X28" s="31">
+      <c r="X28" s="13">
         <f t="shared" si="6"/>
         <v>4.8363402659864385E-2</v>
       </c>
-      <c r="Y28" s="31">
+      <c r="Y28" s="13">
         <f t="shared" si="7"/>
         <v>2.9085556228708065E-2</v>
       </c>
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T29" s="31">
+      <c r="T29" s="13">
         <f t="shared" si="2"/>
         <v>1.0726011326152585E-3</v>
       </c>
-      <c r="U29" s="31">
+      <c r="U29" s="13">
         <f t="shared" si="3"/>
         <v>-4.7009595893940312E-3</v>
       </c>
-      <c r="V29" s="31">
+      <c r="V29" s="13">
         <f t="shared" si="4"/>
         <v>1.178789845857954E-2</v>
       </c>
-      <c r="W29" s="31">
+      <c r="W29" s="13">
         <f t="shared" si="5"/>
         <v>1.2331545464643906E-2</v>
       </c>
-      <c r="X29" s="31">
+      <c r="X29" s="13">
         <f t="shared" si="6"/>
         <v>6.7203509450865118E-2</v>
       </c>
-      <c r="Y29" s="31">
+      <c r="Y29" s="13">
         <f t="shared" si="7"/>
         <v>3.7628630027377041E-2</v>
       </c>
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T30" s="31">
+      <c r="T30" s="13">
         <f t="shared" si="2"/>
         <v>-4.8972228571948458E-4</v>
       </c>
-      <c r="U30" s="31">
+      <c r="U30" s="13">
         <f t="shared" si="3"/>
         <v>-5.2178100793420987E-3</v>
       </c>
-      <c r="V30" s="31">
+      <c r="V30" s="13">
         <f t="shared" si="4"/>
         <v>7.1161220757140556E-3</v>
       </c>
-      <c r="W30" s="31">
+      <c r="W30" s="13">
         <f t="shared" si="5"/>
         <v>2.145602025424935E-2</v>
       </c>
-      <c r="X30" s="31">
+      <c r="X30" s="13">
         <f t="shared" si="6"/>
         <v>5.3121850748457711E-2</v>
       </c>
-      <c r="Y30" s="31">
+      <c r="Y30" s="13">
         <f t="shared" si="7"/>
         <v>3.8358183479932639E-2</v>
       </c>
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T31" s="31">
+      <c r="T31" s="13">
         <f t="shared" si="2"/>
         <v>-1.6191133978591887E-4</v>
       </c>
-      <c r="U31" s="31">
+      <c r="U31" s="13">
         <f t="shared" si="3"/>
         <v>7.3863404524286691E-4</v>
       </c>
-      <c r="V31" s="31">
+      <c r="V31" s="13">
         <f t="shared" si="4"/>
         <v>-4.576913807206151E-3</v>
       </c>
-      <c r="W31" s="31">
+      <c r="W31" s="13">
         <f t="shared" si="5"/>
         <v>-2.7453060663472056E-2</v>
       </c>
-      <c r="X31" s="31">
+      <c r="X31" s="13">
         <f t="shared" si="6"/>
         <v>1.2478955333677488E-2</v>
       </c>
-      <c r="Y31" s="31">
+      <c r="Y31" s="13">
         <f t="shared" si="7"/>
         <v>2.2424507352374223E-2</v>
       </c>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="T32" s="31">
+      <c r="T32" s="13">
         <f t="shared" si="2"/>
         <v>3.2763835042714964E-4</v>
       </c>
-      <c r="U32" s="31">
+      <c r="U32" s="13">
         <f t="shared" si="3"/>
         <v>-5.7683251419953993E-3</v>
       </c>
-      <c r="V32" s="31">
+      <c r="V32" s="13">
         <f t="shared" si="4"/>
         <v>9.8612683599342277E-3</v>
       </c>
-      <c r="W32" s="31">
+      <c r="W32" s="13">
         <f t="shared" si="5"/>
         <v>2.2872080768403247E-2</v>
       </c>
-      <c r="X32" s="31">
+      <c r="X32" s="13">
         <f t="shared" si="6"/>
         <v>6.3356841061008973E-2</v>
       </c>
-      <c r="Y32" s="31">
+      <c r="Y32" s="13">
         <f t="shared" si="7"/>
         <v>3.7839914167488053E-2</v>
       </c>
     </row>
     <row r="33" spans="20:25" x14ac:dyDescent="0.25">
-      <c r="T33" s="31">
+      <c r="T33" s="13">
         <f t="shared" si="2"/>
         <v>3.5051628947257974E-4</v>
       </c>
-      <c r="U33" s="31">
+      <c r="U33" s="13">
         <f t="shared" si="3"/>
         <v>-6.3251123980629306E-3</v>
       </c>
-      <c r="V33" s="31">
+      <c r="V33" s="13">
         <f t="shared" si="4"/>
         <v>1.2023195374459394E-2</v>
       </c>
-      <c r="W33" s="31">
+      <c r="W33" s="13">
         <f t="shared" si="5"/>
         <v>3.0015087212819286E-2</v>
       </c>
-      <c r="X33" s="31">
+      <c r="X33" s="13">
         <f t="shared" si="6"/>
         <v>6.6442767616919279E-2</v>
       </c>
-      <c r="Y33" s="31">
+      <c r="Y33" s="13">
         <f t="shared" si="7"/>
         <v>3.6352825687667525E-2</v>
       </c>
     </row>
     <row r="34" spans="20:25" x14ac:dyDescent="0.25">
-      <c r="T34" s="31"/>
-      <c r="U34" s="31"/>
-      <c r="V34" s="31"/>
-      <c r="W34" s="31"/>
-      <c r="X34" s="31"/>
-      <c r="Y34" s="31"/>
+      <c r="T34" s="13"/>
+      <c r="U34" s="13"/>
+      <c r="V34" s="13"/>
+      <c r="W34" s="13"/>
+      <c r="X34" s="13"/>
+      <c r="Y34" s="13"/>
     </row>
     <row r="35" spans="20:25" x14ac:dyDescent="0.25">
-      <c r="T35" s="31">
+      <c r="T35" s="13">
         <f>_xlfn.STDEV.S(T19:T33)</f>
         <v>1.0671748468220961E-3</v>
       </c>
-      <c r="U35" s="31">
+      <c r="U35" s="13">
         <f t="shared" ref="U35:Y35" si="8">_xlfn.STDEV.S(U19:U33)</f>
         <v>7.8688500421000025E-3</v>
       </c>
-      <c r="V35" s="31">
+      <c r="V35" s="13">
         <f t="shared" si="8"/>
         <v>1.1016145258516748E-2</v>
       </c>
-      <c r="W35" s="31">
+      <c r="W35" s="13">
         <f t="shared" si="8"/>
         <v>7.1179610812383928E-2</v>
       </c>
-      <c r="X35" s="31">
+      <c r="X35" s="13">
         <f t="shared" si="8"/>
         <v>5.2547292552495489E-2</v>
       </c>
-      <c r="Y35" s="31">
+      <c r="Y35" s="13">
         <f t="shared" si="8"/>
         <v>5.3660086491622155E-2</v>
       </c>
     </row>
     <row r="36" spans="20:25" x14ac:dyDescent="0.25">
-      <c r="T36" s="31"/>
-      <c r="U36" s="31"/>
-      <c r="V36" s="31"/>
-      <c r="W36" s="31"/>
-      <c r="X36" s="31"/>
-      <c r="Y36" s="31"/>
+      <c r="T36" s="13"/>
+      <c r="U36" s="13"/>
+      <c r="V36" s="13"/>
+      <c r="W36" s="13"/>
+      <c r="X36" s="13"/>
+      <c r="Y36" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2690,41 +2698,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="24" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="26" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
-      <c r="S1" s="25" t="s">
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="T1" s="25"/>
-      <c r="U1" s="25"/>
+      <c r="T1" s="26"/>
+      <c r="U1" s="26"/>
       <c r="V1" s="6"/>
-      <c r="W1" s="22" t="s">
+      <c r="W1" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
+      <c r="X1" s="23"/>
+      <c r="Y1" s="23"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -4144,41 +4152,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="24" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="26" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
-      <c r="S1" s="25" t="s">
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="T1" s="25"/>
-      <c r="U1" s="25"/>
+      <c r="T1" s="26"/>
+      <c r="U1" s="26"/>
       <c r="V1" s="6"/>
-      <c r="W1" s="22" t="s">
+      <c r="W1" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
+      <c r="X1" s="23"/>
+      <c r="Y1" s="23"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -12783,41 +12791,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="24" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="26" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
-      <c r="S1" s="25" t="s">
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="T1" s="25"/>
-      <c r="U1" s="25"/>
+      <c r="T1" s="26"/>
+      <c r="U1" s="26"/>
       <c r="V1" s="6"/>
-      <c r="W1" s="22" t="s">
+      <c r="W1" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="X1" s="22"/>
-      <c r="Y1" s="22"/>
+      <c r="X1" s="23"/>
+      <c r="Y1" s="23"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -21460,67 +21468,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="27"/>
-      <c r="S1" s="27"/>
-      <c r="T1" s="27"/>
-      <c r="U1" s="27"/>
-      <c r="V1" s="27"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="28"/>
+      <c r="S1" s="28"/>
+      <c r="T1" s="28"/>
+      <c r="U1" s="28"/>
+      <c r="V1" s="28"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="24" t="s">
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="26" t="s">
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="25" t="s">
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+      <c r="S2" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="T2" s="25"/>
-      <c r="U2" s="25"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="26"/>
       <c r="V2" s="6"/>
-      <c r="W2" s="22" t="s">
+      <c r="W2" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="X2" s="22"/>
-      <c r="Y2" s="22"/>
+      <c r="X2" s="23"/>
+      <c r="Y2" s="23"/>
     </row>
     <row r="3" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -27429,67 +27437,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="27"/>
-      <c r="S1" s="27"/>
-      <c r="T1" s="27"/>
-      <c r="U1" s="27"/>
-      <c r="V1" s="27"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="28"/>
+      <c r="S1" s="28"/>
+      <c r="T1" s="28"/>
+      <c r="U1" s="28"/>
+      <c r="V1" s="28"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="24" t="s">
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="26" t="s">
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="25" t="s">
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+      <c r="S2" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="T2" s="25"/>
-      <c r="U2" s="25"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="26"/>
       <c r="V2" s="6"/>
-      <c r="W2" s="22" t="s">
+      <c r="W2" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="X2" s="22"/>
-      <c r="Y2" s="22"/>
+      <c r="X2" s="23"/>
+      <c r="Y2" s="23"/>
     </row>
     <row r="3" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -33398,67 +33406,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="27"/>
-      <c r="S1" s="27"/>
-      <c r="T1" s="27"/>
-      <c r="U1" s="27"/>
-      <c r="V1" s="27"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="28"/>
+      <c r="S1" s="28"/>
+      <c r="T1" s="28"/>
+      <c r="U1" s="28"/>
+      <c r="V1" s="28"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="24" t="s">
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="26" t="s">
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="25" t="s">
+      <c r="O2" s="27"/>
+      <c r="P2" s="27"/>
+      <c r="Q2" s="27"/>
+      <c r="R2" s="27"/>
+      <c r="S2" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="T2" s="25"/>
-      <c r="U2" s="25"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="26"/>
       <c r="V2" s="6"/>
-      <c r="W2" s="22" t="s">
+      <c r="W2" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="X2" s="22"/>
-      <c r="Y2" s="22"/>
+      <c r="X2" s="23"/>
+      <c r="Y2" s="23"/>
     </row>
     <row r="3" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -39844,22 +39852,22 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="30"/>
-      <c r="H1" s="28" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="31"/>
+      <c r="H1" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="31"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -40855,14 +40863,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E12580AD17ADB64691A1BA4C2E042DA4" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6532fc6a52f3455fe895a4f720bca71c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8" xmlns:ns4="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d9a2f75daf18a7097de825f86ff3fec6" ns3:_="" ns4:_="">
     <xsd:import namespace="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
@@ -41115,7 +41115,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -41124,24 +41124,15 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE208467-E14A-4CB9-9FC8-72DFB8E94FF2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{65923CC5-95C4-4597-AADE-A0DCE38786F0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -41160,10 +41151,27 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D595912-0053-4104-933F-CDA3B3DBC546}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE208467-E14A-4CB9-9FC8-72DFB8E94FF2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="c2b20bf0-79f3-4559-a8ab-bcb74dcd8cd8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="08a9f8ec-165a-4165-a8e9-ed45c2de7bcb"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>